<commit_message>
feat: analise paper matéria
</commit_message>
<xml_diff>
--- a/robustez_casos_materia.xlsx
+++ b/robustez_casos_materia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP5"/>
+  <dimension ref="A1:AP6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -774,11 +774,12 @@
       <c r="AO2" t="b">
         <v>1</v>
       </c>
+      <c r="AP2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rho025</t>
+          <t>rho050</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -841,7 +842,7 @@
         <v>0.8</v>
       </c>
       <c r="S3" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="T3" t="n">
         <v>750</v>
@@ -909,11 +910,12 @@
       <c r="AO3" t="b">
         <v>1</v>
       </c>
+      <c r="AP3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rho050</t>
+          <t>rho100</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -976,7 +978,7 @@
         <v>0.8</v>
       </c>
       <c r="S4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="T4" t="n">
         <v>750</v>
@@ -1044,11 +1046,12 @@
       <c r="AO4" t="b">
         <v>1</v>
       </c>
+      <c r="AP4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rho100</t>
+          <t>rho150</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1111,7 +1114,7 @@
         <v>0.8</v>
       </c>
       <c r="S5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="T5" t="n">
         <v>750</v>
@@ -1179,6 +1182,143 @@
       <c r="AO5" t="b">
         <v>1</v>
       </c>
+      <c r="AP5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rho200</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>500</v>
+      </c>
+      <c r="C6" t="n">
+        <v>450</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Circular</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Retangular</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>curta duração</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>madeira natural</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S6" t="n">
+        <v>20</v>
+      </c>
+      <c r="T6" t="n">
+        <v>750</v>
+      </c>
+      <c r="U6" t="n">
+        <v>40</v>
+      </c>
+      <c r="V6" t="n">
+        <v>6</v>
+      </c>
+      <c r="W6" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="X6" t="n">
+        <v>750</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>40</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>50</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>15</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>300</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AM6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="AO6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>